<commit_message>
📊 BIST Screener | 22.05.2026 16:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-22.xlsx
+++ b/data/bist_screener_2026-05-22.xlsx
@@ -9112,7 +9112,7 @@
         <v>10330000</v>
       </c>
       <c r="E199" s="8" t="n">
-        <v>0.4024</v>
+        <v>0.4146</v>
       </c>
       <c r="F199" s="7" t="n">
         <v>69.76000000000001</v>
@@ -25905,34 +25905,38 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>16.18</v>
+        <v>25.02</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0445</v>
+        <v>0.039</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>37920000</v>
-      </c>
-      <c r="E587" s="6" t="inlineStr"/>
+        <v>803570</v>
+      </c>
+      <c r="E587" s="8" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F587" s="7" t="n">
-        <v>45.35</v>
+        <v>40.53</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
       <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="6" t="inlineStr"/>
+      <c r="J587" s="8" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25940,21 +25944,21 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>15.77</v>
+        <v>184.4</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0677</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>38790000</v>
+        <v>7240000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>44.53</v>
+        <v>53.57</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25962,12 +25966,12 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25975,21 +25979,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>69.5</v>
+        <v>13.6</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.09970000000000001</v>
+        <v>0.0709</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>148410</v>
+        <v>25710000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>18.44</v>
+        <v>47.3</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -25997,82 +26001,78 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr"/>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>25.02</v>
+        <v>79.27</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.039</v>
+        <v>-0.0075</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>803570</v>
-      </c>
-      <c r="E590" s="4" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>12060000</v>
+      </c>
+      <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>40.53</v>
+        <v>44.16</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
-      <c r="J590" s="4" t="n">
-        <v>0.6453</v>
-      </c>
-      <c r="K590" s="2" t="inlineStr">
-        <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
-        </is>
-      </c>
+      <c r="J590" s="2" t="inlineStr"/>
+      <c r="K590" s="2" t="inlineStr"/>
+      <c r="L590" s="2" t="inlineStr"/>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>28.54</v>
+        <v>63.7</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.07290000000000001</v>
+        <v>0.0555</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>19000000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>691190</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>54.8</v>
+        <v>47.77</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="J591" s="8" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26080,21 +26080,21 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>39.64</v>
+        <v>15.77</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0999</v>
+        <v>0.0677</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>11650000</v>
+        <v>38790000</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>61.54</v>
+        <v>44.53</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26102,12 +26102,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26115,26 +26115,32 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>17.4</v>
+        <v>5.65</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0351</v>
+        <v>-0.008800000000000001</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>37670000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>21510000</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>33.73</v>
+        <v>46.56</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J593" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26142,7 +26148,7 @@
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26150,29 +26156,33 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>6.01</v>
+        <v>61.3</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0016</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>9290000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>46720</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>44.51</v>
+        <v>30.18</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="J594" s="4" t="n">
+        <v>0.4928</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Taşımacılık</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr"/>
@@ -26181,58 +26191,56 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>61.3</v>
+        <v>173.5</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0016</v>
+        <v>0.0644</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>46720</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>7700000</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>30.18</v>
+        <v>39.68</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="8" t="n">
-        <v>0.4928</v>
-      </c>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>235</v>
+        <v>2.63</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0204</v>
-      </c>
-      <c r="D596" s="5" t="n">
-        <v>10440</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>0.0437</v>
+      </c>
+      <c r="D596" s="3" t="n">
+        <v>130300000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>42.05</v>
+        <v>43.8</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26240,49 +26248,47 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>2.38</v>
+        <v>28.54</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0968</v>
+        <v>0.07290000000000001</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>20400000</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>1</v>
-      </c>
+        <v>19000000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>38.14</v>
+        <v>54.8</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J597" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I597" s="6" t="inlineStr"/>
+      <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26290,21 +26296,23 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>173.5</v>
+        <v>33</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0644</v>
+        <v>0.1</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>7700000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>22390000</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>39.68</v>
+        <v>60.27</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26317,7 +26325,7 @@
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26325,21 +26333,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>2.63</v>
+        <v>69.5</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0437</v>
-      </c>
-      <c r="D599" s="7" t="n">
-        <v>130300000</v>
+        <v>0.09970000000000001</v>
+      </c>
+      <c r="D599" s="9" t="n">
+        <v>148410</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>43.8</v>
+        <v>18.44</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26350,11 +26358,7 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
@@ -26385,56 +26389,58 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>38.88</v>
+        <v>10.55</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.0508</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>5880000</v>
-      </c>
-      <c r="E601" s="6" t="inlineStr"/>
+        <v>674580</v>
+      </c>
+      <c r="E601" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F601" s="7" t="n">
-        <v>45.03</v>
+        <v>62.83</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="I601" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J601" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>73.90000000000001</v>
+        <v>6.01</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0314</v>
+        <v>0.0204</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>30590000</v>
+        <v>9290000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>74.36</v>
+        <v>44.51</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26442,55 +26448,43 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr"/>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>34.3</v>
+        <v>17.4</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.06059999999999999</v>
+        <v>0.0351</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>4780000</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>37670000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>44.54</v>
-      </c>
-      <c r="G603" s="7" t="n">
-        <v>13.56</v>
-      </c>
+        <v>33.73</v>
+      </c>
+      <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26498,58 +26492,56 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>10.55</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0508</v>
+        <v>0.0314</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>674580</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>30590000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>62.83</v>
+        <v>74.36</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J604" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I604" s="2" t="inlineStr"/>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>13.6</v>
+        <v>16.18</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0709</v>
+        <v>0.0445</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>25710000</v>
+        <v>37920000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>47.3</v>
+        <v>45.35</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26557,12 +26549,12 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26570,36 +26562,42 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>33</v>
+        <v>34.3</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.1</v>
+        <v>0.06059999999999999</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>22390000</v>
+        <v>4780000</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.2667</v>
+        <v>0.3528</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>60.27</v>
-      </c>
-      <c r="G606" s="2" t="inlineStr"/>
+        <v>44.54</v>
+      </c>
+      <c r="G606" s="3" t="n">
+        <v>13.56</v>
+      </c>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="2" t="inlineStr"/>
+      <c r="I606" s="4" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J606" s="4" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26607,38 +26605,40 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>63.7</v>
+        <v>127.9</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0555</v>
+        <v>0.0373</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>691190</v>
+        <v>957670</v>
       </c>
       <c r="E607" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.1071</v>
       </c>
       <c r="F607" s="7" t="n">
-        <v>47.77</v>
+        <v>40.21</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="6" t="inlineStr"/>
+      <c r="I607" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
       <c r="J607" s="8" t="n">
-        <v>0.1431</v>
+        <v>-0.4897</v>
       </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26646,40 +26646,40 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>5.65</v>
+        <v>2.38</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>-0.008800000000000001</v>
+        <v>0.0968</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>21510000</v>
+        <v>20400000</v>
       </c>
       <c r="E608" s="4" t="n">
-        <v>0.1672</v>
+        <v>1</v>
       </c>
       <c r="F608" s="3" t="n">
-        <v>46.56</v>
+        <v>38.14</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
       <c r="I608" s="4" t="n">
-        <v>-5.3262</v>
+        <v>-191.6342</v>
       </c>
       <c r="J608" s="4" t="n">
-        <v>-4.2562</v>
+        <v>-0.8093</v>
       </c>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26687,67 +26687,69 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>79.27</v>
+        <v>39.64</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.0075</v>
+        <v>0.0999</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>12060000</v>
+        <v>11650000</v>
       </c>
       <c r="E609" s="6" t="inlineStr"/>
       <c r="F609" s="7" t="n">
-        <v>44.16</v>
+        <v>61.54</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
       <c r="I609" s="6" t="inlineStr"/>
       <c r="J609" s="6" t="inlineStr"/>
-      <c r="K609" s="6" t="inlineStr"/>
-      <c r="L609" s="6" t="inlineStr"/>
+      <c r="K609" s="6" t="inlineStr">
+        <is>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L609" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M609" s="6" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>127.9</v>
+        <v>38.88</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.0373</v>
+        <v>0.06519999999999999</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>957670</v>
-      </c>
-      <c r="E610" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>5880000</v>
+      </c>
+      <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>40.21</v>
+        <v>45.03</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
-      <c r="I610" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J610" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I610" s="2" t="inlineStr"/>
+      <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26755,21 +26757,23 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>184.4</v>
+        <v>235</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.0204</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>7240000</v>
-      </c>
-      <c r="E611" s="6" t="inlineStr"/>
+        <v>10440</v>
+      </c>
+      <c r="E611" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F611" s="7" t="n">
-        <v>53.57</v>
+        <v>42.05</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
@@ -26777,14 +26781,10 @@
       <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L611" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L611" s="6" t="inlineStr"/>
       <c r="M611" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26809,7 +26809,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>22.05.2026 15:30</t>
+          <t>22.05.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 22.05.2026 17:22 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-22.xlsx
+++ b/data/bist_screener_2026-05-22.xlsx
@@ -25905,38 +25905,34 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>25.02</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.039</v>
+        <v>0.0314</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>803570</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>30590000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>40.53</v>
+        <v>74.36</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
       <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="8" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25944,34 +25940,38 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>184.4</v>
+        <v>25.02</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.039</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>7240000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>803570</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>53.57</v>
+        <v>40.53</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="J588" s="4" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25979,21 +25979,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>13.6</v>
+        <v>15.77</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0709</v>
+        <v>0.0677</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>25710000</v>
+        <v>38790000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>47.3</v>
+        <v>44.53</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26001,12 +26001,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26014,65 +26014,77 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>79.27</v>
+        <v>34.3</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0075</v>
+        <v>0.06059999999999999</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>12060000</v>
-      </c>
-      <c r="E590" s="2" t="inlineStr"/>
+        <v>4780000</v>
+      </c>
+      <c r="E590" s="4" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F590" s="3" t="n">
-        <v>44.16</v>
-      </c>
-      <c r="G590" s="2" t="inlineStr"/>
+        <v>44.54</v>
+      </c>
+      <c r="G590" s="3" t="n">
+        <v>13.56</v>
+      </c>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="2" t="inlineStr"/>
-      <c r="J590" s="2" t="inlineStr"/>
-      <c r="K590" s="2" t="inlineStr"/>
-      <c r="L590" s="2" t="inlineStr"/>
+      <c r="I590" s="4" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J590" s="4" t="n">
+        <v>-1.4864</v>
+      </c>
+      <c r="K590" s="2" t="inlineStr">
+        <is>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>63.7</v>
+        <v>184.4</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0555</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>691190</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>7240000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>47.77</v>
+        <v>53.57</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="8" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26080,21 +26092,21 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>15.77</v>
+        <v>38.88</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0677</v>
+        <v>0.06519999999999999</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>38790000</v>
+        <v>5880000</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>44.53</v>
+        <v>45.03</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26102,12 +26114,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26115,40 +26127,38 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>5.65</v>
+        <v>63.7</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.008800000000000001</v>
+        <v>0.0555</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>21510000</v>
+        <v>691190</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>46.56</v>
+        <v>47.77</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
+      <c r="I593" s="6" t="inlineStr"/>
       <c r="J593" s="8" t="n">
-        <v>-4.2562</v>
+        <v>0.1431</v>
       </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26156,69 +26166,75 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>61.3</v>
+        <v>28.54</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0016</v>
+        <v>0.07290000000000001</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>46720</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>19000000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>30.18</v>
+        <v>54.8</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="4" t="n">
-        <v>0.4928</v>
-      </c>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr"/>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>173.5</v>
+        <v>2.38</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0644</v>
+        <v>0.0968</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>7700000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>20400000</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>39.68</v>
+        <v>38.14</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="I595" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J595" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26226,69 +26242,77 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>2.63</v>
+        <v>10.55</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0437</v>
-      </c>
-      <c r="D596" s="3" t="n">
-        <v>130300000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>0.0508</v>
+      </c>
+      <c r="D596" s="5" t="n">
+        <v>674580</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>43.8</v>
+        <v>62.83</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J596" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr"/>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>28.54</v>
+        <v>127.9</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.07290000000000001</v>
+        <v>0.0373</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>19000000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>957670</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>54.8</v>
+        <v>40.21</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26333,21 +26357,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>69.5</v>
+        <v>6.01</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.09970000000000001</v>
+        <v>0.0204</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>148410</v>
+        <v>9290000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>18.44</v>
+        <v>44.51</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26364,83 +26388,93 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>EKDMR</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>49.5</v>
-      </c>
-      <c r="C600" s="2" t="inlineStr"/>
-      <c r="D600" s="2" t="inlineStr"/>
+        <v>69.5</v>
+      </c>
+      <c r="C600" s="4" t="n">
+        <v>0.09970000000000001</v>
+      </c>
+      <c r="D600" s="5" t="n">
+        <v>148410</v>
+      </c>
       <c r="E600" s="2" t="inlineStr"/>
-      <c r="F600" s="2" t="inlineStr"/>
+      <c r="F600" s="3" t="n">
+        <v>18.44</v>
+      </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="2" t="inlineStr"/>
       <c r="J600" s="2" t="inlineStr"/>
-      <c r="K600" s="2" t="inlineStr"/>
-      <c r="L600" s="2" t="inlineStr">
-        <is>
-          <t>BIST TÜM</t>
-        </is>
-      </c>
+      <c r="K600" s="2" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr"/>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>10.55</v>
+        <v>5.65</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0508</v>
+        <v>-0.008800000000000001</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>674580</v>
+        <v>21510000</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.95</v>
+        <v>0.1672</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>62.83</v>
+        <v>46.56</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-5.3262</v>
       </c>
       <c r="J601" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-4.2562</v>
       </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>6.01</v>
+        <v>16.18</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0445</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>9290000</v>
+        <v>37920000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>44.51</v>
+        <v>45.35</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26448,30 +26482,34 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>17.4</v>
+        <v>2.63</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0351</v>
-      </c>
-      <c r="D603" s="9" t="n">
-        <v>37670000</v>
+        <v>0.0437</v>
+      </c>
+      <c r="D603" s="7" t="n">
+        <v>130300000</v>
       </c>
       <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>33.73</v>
+        <v>43.8</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26484,7 +26522,7 @@
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26492,21 +26530,21 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>73.90000000000001</v>
+        <v>39.64</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0314</v>
+        <v>0.0999</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>30590000</v>
+        <v>11650000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>74.36</v>
+        <v>61.54</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26514,12 +26552,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26527,34 +26565,24 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>EKDMR</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>16.18</v>
-      </c>
-      <c r="C605" s="8" t="n">
-        <v>0.0445</v>
-      </c>
-      <c r="D605" s="9" t="n">
-        <v>37920000</v>
-      </c>
+        <v>49.5</v>
+      </c>
+      <c r="C605" s="6" t="inlineStr"/>
+      <c r="D605" s="6" t="inlineStr"/>
       <c r="E605" s="6" t="inlineStr"/>
-      <c r="F605" s="7" t="n">
-        <v>45.35</v>
-      </c>
+      <c r="F605" s="6" t="inlineStr"/>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
       <c r="J605" s="6" t="inlineStr"/>
-      <c r="K605" s="6" t="inlineStr">
-        <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
+      <c r="K605" s="6" t="inlineStr"/>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TÜM</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26562,42 +26590,34 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>34.3</v>
+        <v>173.5</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.06059999999999999</v>
+        <v>0.0644</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>4780000</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>7700000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>44.54</v>
-      </c>
-      <c r="G606" s="3" t="n">
-        <v>13.56</v>
-      </c>
+        <v>39.68</v>
+      </c>
+      <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26605,40 +26625,34 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>127.9</v>
+        <v>13.6</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0373</v>
+        <v>0.0709</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>957670</v>
-      </c>
-      <c r="E607" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>25710000</v>
+      </c>
+      <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>40.21</v>
+        <v>47.3</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J607" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I607" s="6" t="inlineStr"/>
+      <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26646,62 +26660,50 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>2.38</v>
+        <v>79.27</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0968</v>
+        <v>-0.0075</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>20400000</v>
-      </c>
-      <c r="E608" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>12060000</v>
+      </c>
+      <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>38.14</v>
+        <v>44.16</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
-      <c r="I608" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J608" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
-      <c r="K608" s="2" t="inlineStr">
-        <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L608" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+      <c r="I608" s="2" t="inlineStr"/>
+      <c r="J608" s="2" t="inlineStr"/>
+      <c r="K608" s="2" t="inlineStr"/>
+      <c r="L608" s="2" t="inlineStr"/>
       <c r="M608" s="2" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>39.64</v>
+        <v>235</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0999</v>
+        <v>0.0204</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>11650000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>10440</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>61.54</v>
+        <v>42.05</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
@@ -26709,34 +26711,30 @@
       <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L609" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L609" s="6" t="inlineStr"/>
       <c r="M609" s="6" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>38.88</v>
+        <v>17.4</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.0351</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>5880000</v>
+        <v>37670000</v>
       </c>
       <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>45.03</v>
+        <v>33.73</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26744,12 +26742,12 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26757,31 +26755,33 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>235</v>
+        <v>61.3</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0.0204</v>
+        <v>0.0016</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>10440</v>
+        <v>46720</v>
       </c>
       <c r="E611" s="8" t="n">
-        <v>0.2578</v>
+        <v>0.58</v>
       </c>
       <c r="F611" s="7" t="n">
-        <v>42.05</v>
+        <v>30.18</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
       <c r="I611" s="6" t="inlineStr"/>
-      <c r="J611" s="6" t="inlineStr"/>
+      <c r="J611" s="8" t="n">
+        <v>0.4928</v>
+      </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Taşımacılık</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr"/>
@@ -26809,7 +26809,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>22.05.2026 16:30</t>
+          <t>22.05.2026 17:22</t>
         </is>
       </c>
     </row>

</xml_diff>